<commit_message>
Add fail-closed ds006072 validation gate
</commit_message>
<xml_diff>
--- a/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
+++ b/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
@@ -118,7 +118,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Drug-order mapping and unchanged scoring are locked, but local ds006072 CIFTI/module time-series payloads are absent. Download or provide authorized processed rest CIFTIs before claiming validation.</t>
+          <t>No paired ds006072 empirical-viewer subject views exist. Provide harmonized records under results/psilocybin_ds006072/empirical_viewer/subject_views with ses-PLCB control and ses-LSD psilocybin aliases.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -128,7 +128,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>extraction_contract_ready_missing_local_cifti_payloads</t>
+          <t>blocked_missing_local_ds006072_empirical_viewer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>extraction_contract_ready_missing_local_cifti_payloads</t>
+          <t>blocked_missing_local_ds006072_empirical_viewer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ds006072 CIFTI external validation extraction
</commit_message>
<xml_diff>
--- a/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
+++ b/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
@@ -118,7 +118,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No paired ds006072 empirical-viewer subject views exist. Provide harmonized records under results/psilocybin_ds006072/empirical_viewer/subject_views with ses-PLCB control and ses-LSD psilocybin aliases.</t>
+          <t>Comparable ranking generated.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -128,7 +128,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>blocked_missing_local_ds006072_empirical_viewer</t>
+          <t>implemented_ds006072_unchanged_scoring_validation</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>blocked_missing_local_ds006072_empirical_viewer</t>
+          <t>implemented_ds006072_unchanged_scoring_validation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preserve derived artifacts in Pages build
</commit_message>
<xml_diff>
--- a/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
+++ b/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
@@ -118,7 +118,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No paired ds006072 empirical-viewer subject views exist. Provide harmonized records under results/psilocybin_ds006072/empirical_viewer/subject_views with ses-PLCB control and ses-LSD psilocybin aliases.</t>
+          <t>Comparable ranking generated.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -128,7 +128,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>blocked_missing_local_ds006072_empirical_viewer</t>
+          <t>implemented_ds006072_unchanged_scoring_validation</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>blocked_missing_local_ds006072_empirical_viewer</t>
+          <t>implemented_ds006072_unchanged_scoring_validation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden dashboard feature audit
</commit_message>
<xml_diff>
--- a/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
+++ b/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
@@ -246,7 +246,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>None/None measurable proxy checks aligned.</t>
+          <t>4/6 measurable proxy checks aligned.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>blocked_no_measurable_literature_checks</t>
+          <t>requires_mismatch_diagnosis_2_of_6_checks</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,846 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
-    <row r="1"/>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>graph_control</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>graph_source</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>lsd_vs_placebo_receptor_transition_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>receptor_vs_random_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>receptor_vs_uniform_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>rewire_index</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>state_target_alignment_receptor</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>support_score</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>macro_proxy_graph</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>macro_proxy_graph; proxy graph control, not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4.702198506533535</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-14.214731114495072</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>-34.3869884708404</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.21183035701941078</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>uniform_weight_graph</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>uniform_weight_graph; proxy graph control, not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3.8943761126499026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>-3.803757951899512</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>-22.24847009578297</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.31552330412219354</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>degree_expected_graph</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>degree_expected_graph; proxy graph control, not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4.470415240659168</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-9.71664619458491</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-29.29573443489324</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.26147021938726467</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3.4953301013006044</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3.872719827893189</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-12.221300137231095</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.44131554549238816</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>4.926186697188426</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-0.7328999224900453</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-17.97723417118442</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.42589749866565585</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3.082625519020206</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>7.7947726892359315</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-10.193289417449455</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.4983398321844616</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5.104717448180986</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-22.78673100971311</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>-43.01623602104077</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.15207428819066632</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4.495686968120134</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-8.923383183222825</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>-27.53279803714942</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.28951678007923065</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3.350800119672593</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>-0.9532812810829832</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-19.910991163435906</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.3530642939818865</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4.046499086247285</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>-4.162754862386243</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>-22.62151821545653</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.3076519162322807</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>4.013860098578283</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>-8.335725281188644</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-29.89037925952308</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.2754265146030591</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>4.8005011010202265</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-4.654984828636728</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-22.587316306527363</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.33073733344921175</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>4.464124957810071</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-13.855651262170744</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-32.861072589957736</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.23198197109099977</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>4.29996007221886</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>-1.639990479219674</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>-19.076950180867062</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.34230743372875594</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>4.4466356917017</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>-15.636000165679254</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>-34.244904784852</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.19075149371575462</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>4.487833965521429</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-15.885659635150416</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>-33.09941121308414</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.19967631618440163</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>3.890688463314012</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>-6.353141958519869</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>-24.966835315844833</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.30270786659692056</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>3.3460787238893253</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-7.191985415964259</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>-27.165905550833298</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.19790713924521625</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>edge_weight_rewire_null</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>rewired macro-proxy edge-weight null; not HCP structural connectome</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4.3178379982059845</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>-6.439744614853897</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>-24.950712439624514</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0.2994188224961803</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1511,7 +2350,339 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
-    <row r="1"/>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>claim_status</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>expected_direction</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>mean_delta</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>null_family</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>prior_source</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>signed_effect_size</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>proxy_only_not_pet_receptor_claim</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>positive means LSD within-condition transitions need less receptor-profile control energy than placebo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4.702198506533535</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>lsd_vs_placebo_receptor_transition_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>coarse_receptor_proxy</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>coarse module-level proxy prior from receptor-gradient model config; not a PET-derived receptor map</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.37576604844255507</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>proxy_only_not_pet_receptor_claim</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>positive means LSD within-condition transitions need less uniform-control energy than placebo</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6.935892752544529</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>lsd_vs_placebo_uniform_transition_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>uniform_control</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>coarse module-level proxy prior from receptor-gradient model config; not a PET-derived receptor map</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.7242170950688606</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>proxy_only_not_pet_receptor_claim</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>positive means receptor-prior control needs less energy than uniform control</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-34.3869884708404</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>receptor_vs_uniform_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>uniform_control</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>coarse module-level proxy prior from receptor-gradient model config; not a PET-derived receptor map</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-1.457887579613032</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>proxy_only_not_pet_receptor_claim</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>positive means receptor-prior control needs less energy than random receptor-prior permutations</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>-15.4342613806409</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>receptor_vs_random_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>random_permutation</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>coarse module-level proxy prior from receptor-gradient model config; not a PET-derived receptor map</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>-0.8321254106889895</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>proxy_only_not_pet_receptor_claim</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>positive means hierarchy-prior control needs less energy than uniform control</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>-300.46956304822345</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>hierarchy_vs_uniform_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>uniform_control</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>coarse module-level proxy prior from receptor-gradient model config; not a PET-derived receptor map</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-2.2969792663885165</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>proxy_only_not_pet_receptor_claim</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>positive means transmodal-prior control needs less energy than uniform control</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-674.315980973865</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>transmodal_vs_uniform_energy_reduction_pct</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>uniform_control</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>coarse module-level proxy prior from receptor-gradient model config; not a PET-derived receptor map</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-2.0346717830255048</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>proxy_only_not_pet_receptor_claim</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>positive means modules with higher receptor prior align with larger LSD-minus-placebo state displacement</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.13300315069221882</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>state_target_alignment_receptor</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>coarse_receptor_proxy</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>coarse module-level proxy prior from receptor-gradient model config; not a PET-derived receptor map</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.46364101084434517</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>blocked_until_neuromaps_or_FS5ht_projection_exists</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PET-derived receptor map should outperform spatial nulls</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>spatial_autocorrelation_preserving_null</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>spatial_null_missing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>missing PET receptor map</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync thesis gate status artifacts
</commit_message>
<xml_diff>
--- a/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
+++ b/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
@@ -373,7 +373,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>planned comparison</t>
+          <t>implemented directional proxy benchmark</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>planned biological prior</t>
+          <t>implemented PET receptor-prior sensitivity</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>planned graph prior</t>
+          <t>implemented HCP structural graph sensitivity</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>planned parcellation</t>
+          <t>implemented Schaefer/Yeo sensitivity</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">

</xml_diff>

<commit_message>
Revamp thesis dashboard evidence loop
</commit_message>
<xml_diff>
--- a/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
+++ b/results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx
@@ -109,27 +109,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>results/psilocybin_ds006072/</t>
+          <t>results/confound_controls/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t/>
+          <t>Local repo search, OpenNeuro ds003059 snapshot metadata, and public OpenNeuroDerivatives repo checks did not verify subject-level FD/DVARS/censoring confounds.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>parcellation_matched_schaefer100_yeo7_external_validation; ranking_differs_from_lsd_top_layer; ds006072 top=E, LSD reference top=C.</t>
+          <t>Schaefer/Yeo C sensitivity exists, but final C claims remain gated because strict subject/run FD/DVARS/censoring confounds are not proof-ready or high-burden exclusions are unstable.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Psilocybin ds006072</t>
+          <t>Motion-sensitive C gate</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>implemented_ds006072_unchanged_scoring_validation</t>
+          <t>blocked_motion_sensitive_c_claim_requires_authorized_confound_exclusions</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -141,7 +141,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>results/structural_connectome/</t>
+          <t>results/psilocybin_ds006072/</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -151,17 +151,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Structural graph sensitivity generated.</t>
+          <t>parcellation_matched_schaefer100_yeo7_external_validation; ranking_differs_from_lsd_top_layer; ds006072 top=E, LSD reference top=C.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>HCP structural graph</t>
+          <t>Psilocybin ds006072</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>implemented_hcp_structural_graph_sensitivity</t>
+          <t>implemented_ds006072_unchanged_scoring_validation</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -173,7 +173,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>results/receptor_priors/</t>
+          <t>results/structural_connectome/</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -183,17 +183,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PET receptor sensitivity generated.</t>
+          <t>Structural graph sensitivity generated; rewires=implemented_hcp_structural_graph_rewire_nulls.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PET receptor priors</t>
+          <t>HCP structural graph</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>implemented_pet_receptor_prior_sensitivity</t>
+          <t>implemented_hcp_structural_graph_sensitivity</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -205,7 +205,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>results/parcellation_sensitivity/</t>
+          <t>results/receptor_priors/</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -215,17 +215,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Status matrix generated; see per-parcellation rows.</t>
+          <t>PET receptor sensitivity generated; claim gate=not_supported_after_pet_spatial_nulls.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Schaefer/Yeo sensitivity</t>
+          <t>PET receptor priors</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>implemented_status_matrix</t>
+          <t>implemented_pet_receptor_prior_sensitivity</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -237,32 +237,64 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>results/parcellation_sensitivity/</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Status matrix generated; see per-parcellation rows.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Schaefer/Yeo sensitivity</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>implemented_status_matrix</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>results/literature_benchmark/</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>4/6 measurable proxy checks aligned.</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5/7 measurable proxy checks aligned. Striatal gate=implemented_striatal_unimodal_proxy_benchmark.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Mega-analysis comparison</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>implemented_directional_proxy_benchmark</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -809,12 +841,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C survives Schaefer/Yeo 100/200 and Yeo 7/17 with comparable direction</t>
+          <t>C final thesis claim passes motion-sensitive exclusions</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ds003059 parcellation sensitivity artifacts</t>
+          <t>ds003059 run-01/run-03 plus motion/confound control artifacts</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -824,267 +856,361 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Schaefer 100/200 and Yeo 7/17 versus the current 8-module proxy</t>
+          <t>subject/run FD, DVARS, censoring/outlier burden, image-QC, and high-burden exclusions</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>parcellation_sensitivity_table</t>
+          <t>motion_confound_control_table; module_dvars_control_table; image_motion_qc_table</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>results/parcellation_sensitivity/parcellation_status.csv; results/parcellation_sensitivity/parcellation_ranking_comparison.csv; results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx</t>
+          <t>results/confound_controls/motion_confound_control_status.json; results/confound_controls/module_dvars_control_status.json; results/confound_controls/image_motion_qc_status.json</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Schaefer et al. 2018 Cerebral Cortex https://doi.org/10.1093/cercor/bhx179</t>
+          <t>Carhart-Harris et al. 2016 PNAS https://doi.org/10.1073/pnas.1518377113</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Status matrix is not full sensitivity evidence unless parcellation-specific empirical viewer and ranking rows exist.</t>
+          <t>Current local checkout lacks authorized subject/run fMRIPrep FD, DVARS, and censoring confounds; image-derived or published aggregate QC cannot complete the strict gate.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>implemented_c_top_rank_all_requested_parcellations</t>
+          <t>blocked_motion_sensitive_c_claim_requires_authorized_confound_exclusions</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E survives real structural-connectome graph</t>
+          <t>C survives Schaefer/Yeo 100/200 and Yeo 7/17 with comparable direction</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HCP Young Adult or local normative structural-connectome CSV</t>
+          <t>ds003059 parcellation sensitivity artifacts</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>E network-control energy</t>
+          <t>C hierarchy/routing</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>macro proxy graph; uniform graph; degree-expected graph; edge-weight rewires</t>
+          <t>Schaefer 100/200 and Yeo 7/17 versus the current 8-module proxy</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>dynamic_control_plot; structural_proxy_null_table</t>
+          <t>parcellation_sensitivity_table</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>results/structural_connectome/structural_connectome_status.json; results/structural_connectome/proxy_graph_control_nulls.csv</t>
+          <t>results/parcellation_sensitivity/parcellation_status.csv; results/parcellation_sensitivity/parcellation_ranking_comparison.csv; results/thesis_evidence_loop/exports/thesis_evidence_loop_tables.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>HCP Young Adult https://www.humanconnectome.org/study/hcp-young-adult; Singleton et al. 2022 Nature Communications https://www.nature.com/articles/s41467-022-33578-1</t>
+          <t>Schaefer et al. 2018 Cerebral Cortex https://doi.org/10.1093/cercor/bhx179</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Blocked unless HCP/normative structural graph CSV exists; proxy graph controls are not structural-connectome evidence.</t>
+          <t>Status matrix is not full sensitivity evidence unless parcellation-specific empirical viewer and ranking rows exist.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>implemented_hcp_structural_graph_sensitivity</t>
+          <t>implemented_c_top_rank_all_requested_parcellations</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E survives PET receptor-map priors</t>
+          <t>E survives real structural-connectome graph</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>neuromaps/FS5ht 5-HT2A PET receptor prior projected to modules</t>
+          <t>HCP Young Adult or local normative structural-connectome CSV</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>E receptor-informed network-control energy</t>
+          <t>E network-control energy</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>uniform; random permutation; degree control; spatial/autocorrelation null</t>
+          <t>macro proxy graph; uniform graph; degree-expected graph; edge-weight rewires</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>dynamic_control_plot; receptor_null_table</t>
+          <t>dynamic_control_plot; structural_proxy_null_table</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>results/receptor_priors/receptor_prior_status.json; results/receptor_priors/proxy_receptor_null_board.csv</t>
+          <t>results/structural_connectome/structural_connectome_status.json; results/structural_connectome/proxy_graph_control_nulls.csv</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Markello et al. 2022 Nature Methods https://www.nature.com/articles/s41592-022-01625-w; Singleton et al. 2022 Nature Communications https://www.nature.com/articles/s41467-022-33578-1</t>
+          <t>HCP Young Adult https://www.humanconnectome.org/study/hcp-young-adult; Singleton et al. 2022 Nature Communications https://www.nature.com/articles/s41467-022-33578-1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Blocked unless PET-derived receptor prior and spatial nulls exist; current receptor board is a coarse proxy.</t>
+          <t>Structural graph sensitivity is still a normative/proxy sensitivity layer; graph-rewire nulls test topology dependence but do not establish biological causality.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>implemented_pet_receptor_prior_sensitivity</t>
+          <t>implemented_hcp_structural_graph_sensitivity</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ds006072 psilocybin tests the LSD A+B+C+D+E ranking</t>
+          <t>E survives PET receptor-map priors</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OpenNeuro ds006072 psilocybin precision functional mapping</t>
+          <t>neuromaps/FS5ht 5-HT2A PET receptor prior projected to modules</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A+B+C+D+E mechanism ranking</t>
+          <t>E receptor-informed network-control energy</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>same scoring rules as LSD; paired psilocybin/control empirical viewer</t>
+          <t>uniform; random permutation; degree control; spatial/autocorrelation null</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>thesis_loop_steps; LSD-vs-psilocybin ranking comparison</t>
+          <t>dynamic_control_plot; receptor_null_table</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>results/psilocybin_ds006072/psilocybin_ds006072_status.json; results/thesis_evidence_loop/exports/ds006072_summary.csv</t>
+          <t>results/receptor_priors/receptor_prior_status.json; results/receptor_priors/proxy_receptor_null_board.csv</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dosenbach/Siegel group 2025 Scientific Data https://doi.org/10.1038/s41597-025-05189-0; OpenNeuro ds006072 https://openneuro.org/datasets/ds006072</t>
+          <t>Markello et al. 2022 Nature Methods https://www.nature.com/articles/s41592-022-01625-w; Singleton et al. 2022 Nature Communications https://www.nature.com/articles/s41467-022-33578-1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Comparable Schaefer100/Yeo7 scoring is a cross-drug stress test; a differing top layer is negative/partial external evidence, not replication.</t>
+          <t>PET-derived 5-HT2A priors and Schaefer100 Moran spatial nulls are required together; current spatial-null/FDR evidence blocks receptor-claim promotion if support is absent.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>implemented_ds006072_unchanged_scoring_validation</t>
+          <t>not_supported_after_pet_spatial_nulls</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Final C/D/E pattern aligns with psychedelic mega-analysis and NCT anchors</t>
+          <t>ds006072 psilocybin tests the LSD A+B+C+D+E ranking</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ds003059 LSD proxy deltas plus literature benchmark rows</t>
+          <t>OpenNeuro ds006072 psilocybin precision functional mapping</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>C hierarchy/routing; D dynamic repertoire; E network-control energy</t>
+          <t>A+B+C+D+E mechanism ranking</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>directional proxy benchmark; explicit mismatches retained</t>
+          <t>same scoring rules as LSD; paired psilocybin/control empirical viewer</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>literature_benchmark_plot; literature_benchmark_table</t>
+          <t>thesis_loop_steps; LSD-vs-psilocybin ranking comparison</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>results/literature_benchmark/literature_benchmark.csv; results/thesis_evidence_loop/claim_evidence_matrix.csv</t>
+          <t>results/psilocybin_ds006072/psilocybin_ds006072_status.json; results/thesis_evidence_loop/exports/ds006072_summary.csv</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Girn et al. 2026 Nature Medicine https://www.nature.com/articles/s41591-026-04287-9; Singleton et al. 2022 Nature Communications https://www.nature.com/articles/s41467-022-33578-1</t>
+          <t>Dosenbach/Siegel group 2025 Scientific Data https://doi.org/10.1038/s41597-025-05189-0; OpenNeuro ds006072 https://openneuro.org/datasets/ds006072</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Directional proxy benchmark only; not a mega-analysis or full NCT reproduction.</t>
+          <t>Comparable Schaefer100/Yeo7 scoring is a cross-drug stress test; a differing top layer is negative/partial external evidence, not replication.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>implemented_directional_proxy_benchmark</t>
+          <t>implemented_ds006072_unchanged_scoring_validation</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Final C/D/E pattern aligns with psychedelic mega-analysis and NCT anchors</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ds003059 LSD proxy deltas plus literature benchmark rows</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>C hierarchy/routing; D dynamic repertoire; E network-control energy</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>directional proxy benchmark; explicit mismatches retained</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>literature_benchmark_plot; literature_benchmark_table</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>results/literature_benchmark/literature_benchmark.csv; results/thesis_evidence_loop/claim_evidence_matrix.csv</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Girn et al. 2026 Nature Medicine https://www.nature.com/articles/s41591-026-04287-9; Singleton et al. 2022 Nature Communications https://www.nature.com/articles/s41467-022-33578-1</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Directional proxy benchmark only; not a mega-analysis or full NCT reproduction.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>implemented_directional_proxy_benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nature Medicine striatal-unimodal benchmark is testable</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ds003059/ds006072 high-resolution parcellation benchmark rows</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>C/D striatal-subcortical routing</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>dedicated caudate/putamen/accumbens parcels versus cortical-only proxy rows</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>literature_benchmark_table; Schaefer100/Yeo7 + Harvard-Oxford striatal sensitivity row</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>results/literature_benchmark/literature_benchmark.csv; results/thesis_evidence_loop/claim_evidence_matrix.csv</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Girn et al. 2026 Nature Medicine https://www.nature.com/articles/s41591-026-04287-9</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>The current implemented row uses bilateral Harvard-Oxford striatum as a proxy. It tests whether the benchmark is directionally measurable, not whether the Nature Medicine nucleus-level result is reproduced.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>implemented_striatal_unimodal_proxy_benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Failed literature checks are diagnosed as contradiction or proxy mismatch</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>results/literature_benchmark/literature_benchmark.csv</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>C/D/E failure-case analysis</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>row-level mismatch review; sign/opposes/weak checks</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>literature_benchmark_table</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>results/literature_benchmark/literature_benchmark.csv; results/thesis_evidence_loop/claim_evidence_matrix.csv</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Girn et al. 2026 Nature Medicine https://www.nature.com/articles/s41591-026-04287-9; Singleton et al. 2022 Nature Communications https://www.nature.com/articles/s41467-022-33578-1</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Requires explicit per-row mismatch reason; unresolved mismatches stay out of final conclusions.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>requires_mismatch_diagnosis_2_of_6_checks</t>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>requires_mismatch_diagnosis_2_of_7_checks</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1430,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_7</t>
+          <t>schaefer_100_yeo_7_striatal</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1319,7 +1445,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>results/parcellation_sensitivity/schaefer_200_yeo_7/summary.json</t>
+          <t>results/parcellation_sensitivity/schaefer_100_yeo_7_striatal/summary.json</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1336,7 +1462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>schaefer_100_yeo_17</t>
+          <t>schaefer_200_yeo_7</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1351,7 +1477,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>results/parcellation_sensitivity/schaefer_100_yeo_17/summary.json</t>
+          <t>results/parcellation_sensitivity/schaefer_200_yeo_7/summary.json</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1368,25 +1494,57 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>schaefer_100_yeo_17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>implemented_mechanism_ranking</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>results/parcellation_sensitivity/schaefer_100_yeo_17/summary.json</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>schaefer_200_yeo_17</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>implemented_mechanism_ranking</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>results/parcellation_sensitivity/schaefer_200_yeo_17/summary.json</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1569,7 +1727,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_7</t>
+          <t>schaefer_100_yeo_7_striatal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1579,7 +1737,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.3812357350841233</t>
+          <t>0.47213485004447986</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1596,7 +1754,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_7</t>
+          <t>schaefer_100_yeo_7_striatal</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1606,7 +1764,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.27924167039914227</t>
+          <t>0.42763493354223536</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1623,7 +1781,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_7</t>
+          <t>schaefer_100_yeo_7_striatal</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1633,7 +1791,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.16163290115024492</t>
+          <t>0.1883308443884962</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1650,7 +1808,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_7</t>
+          <t>schaefer_100_yeo_7_striatal</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1660,7 +1818,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.0534825202256326</t>
+          <t>0.1769569077988587</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1677,7 +1835,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_7</t>
+          <t>schaefer_100_yeo_7_striatal</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1687,7 +1845,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-3.866778980018167</t>
+          <t>-1.5955788116726106</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1704,7 +1862,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>schaefer_100_yeo_17</t>
+          <t>schaefer_200_yeo_7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1714,7 +1872,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.38838412413825185</t>
+          <t>0.3812357350841233</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1731,7 +1889,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>schaefer_100_yeo_17</t>
+          <t>schaefer_200_yeo_7</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1741,7 +1899,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.38076368940200545</t>
+          <t>0.27924167039914227</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1753,12 +1911,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>schaefer_100_yeo_17</t>
+          <t>schaefer_200_yeo_7</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1768,24 +1926,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.14146425621619316</t>
+          <t>0.16163290115024492</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>implemented_proxy_control_energy</t>
+          <t>implemented_first_pass</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>schaefer_100_yeo_17</t>
+          <t>schaefer_200_yeo_7</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1795,12 +1953,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.14070315698857125</t>
+          <t>0.0534825202256326</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>implemented_first_pass</t>
+          <t>implemented_proxy_control_energy</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1970,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>schaefer_100_yeo_17</t>
+          <t>schaefer_200_yeo_7</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1822,7 +1980,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.5587841629062331</t>
+          <t>-3.866778980018167</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1839,7 +1997,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_17</t>
+          <t>schaefer_100_yeo_17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1849,7 +2007,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.3890043610256203</t>
+          <t>0.38838412413825185</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1866,7 +2024,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_17</t>
+          <t>schaefer_100_yeo_17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1876,7 +2034,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.3238425854807948</t>
+          <t>0.38076368940200545</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1888,12 +2046,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_17</t>
+          <t>schaefer_100_yeo_17</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1903,24 +2061,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.16163290115024492</t>
+          <t>0.14146425621619316</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>implemented_first_pass</t>
+          <t>implemented_proxy_control_energy</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>schaefer_200_yeo_17</t>
+          <t>schaefer_100_yeo_17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1930,12 +2088,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.034502729231533</t>
+          <t>0.14070315698857125</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>implemented_proxy_control_energy</t>
+          <t>implemented_first_pass</t>
         </is>
       </c>
     </row>
@@ -1947,20 +2105,155 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>schaefer_100_yeo_17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>-1.5587841629062331</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>implemented_negative_control_baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>schaefer_200_yeo_17</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0.3890043610256203</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>implemented_first_pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>schaefer_200_yeo_17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0.3238425854807948</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>implemented_first_pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>schaefer_200_yeo_17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0.16163290115024492</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>implemented_first_pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>schaefer_200_yeo_17</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0.034502729231533</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>implemented_proxy_control_energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>schaefer_200_yeo_17</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>-3.8667789800181773</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>implemented_negative_control_baseline</t>
         </is>

</xml_diff>